<commit_message>
chore: Update database and Excel master sheets with latest student results
</commit_message>
<xml_diff>
--- a/Extra_curricular/2025_2026/Second_term/JSS3/extra_jss3_second_term_2025_2026.xlsx
+++ b/Extra_curricular/2025_2026/Second_term/JSS3/extra_jss3_second_term_2025_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Reporter\Extra_curricular\2025_2026\Second_term\JSS3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C7875B2-D9D4-4402-8DE3-0860E1BE8764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B633460B-006A-4577-8EE3-485718ACB915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{A3584512-35F2-4ADB-935B-FFA0649CF8D6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="39">
   <si>
     <t>Admission_no</t>
   </si>
@@ -57,9 +57,6 @@
     <t>Discipline</t>
   </si>
   <si>
-    <t>you have proven to be a great student I wish you more success in your endeavours</t>
-  </si>
-  <si>
     <t>TEST</t>
   </si>
   <si>
@@ -96,33 +93,18 @@
     <t>reason</t>
   </si>
   <si>
-    <t>holiday</t>
-  </si>
-  <si>
     <t>next_term</t>
   </si>
   <si>
-    <t>Press Club</t>
-  </si>
-  <si>
     <t>Girls Guide</t>
   </si>
   <si>
     <t>JETS Club</t>
   </si>
   <si>
-    <t>Sex Edu Club</t>
-  </si>
-  <si>
     <t>Red Cross</t>
   </si>
   <si>
-    <t>Farmers Club</t>
-  </si>
-  <si>
-    <t>English Club</t>
-  </si>
-  <si>
     <t>Boys Scout</t>
   </si>
   <si>
@@ -133,14 +115,49 @@
   </si>
   <si>
     <t>4th, May 2026</t>
+  </si>
+  <si>
+    <t>nil</t>
+  </si>
+  <si>
+    <t>Congratulations !!!!! For the Conlusion of your Second term/B.E.C.E mock Examinations</t>
+  </si>
+  <si>
+    <t>Congratulations !!!!! For the Conlusion of your Second term/B.E.C.E mock Examinations, But have at the back of your mind that this is not the beginning, the journey is just starting, I would really urge you to work more on you punctuality and be very much active and cooperative in your class and Academic Operations</t>
+  </si>
+  <si>
+    <t>Congratulations !!!!! For the Conlusion of your Second term/B.E.C.E mock Examinations, But have at the back of your mind that this is not the beginning, the journey is just starting, I will be expecting to meet you at the top next time</t>
+  </si>
+  <si>
+    <t>Congratulations !!!!! For the Conlusion of your Second term/B.E.C.E mock Examinations, Your Performance has shown that you do something Worthful Independently congratulations again.</t>
+  </si>
+  <si>
+    <t>Congratulations !!!!! For the Conlusion of your Second term/B.E.C.E mock Examinations, this is a Wonderful performance I want to see you ace all subjects next time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Congratulations !!!!! For the Conlusion of your Second term/B.E.C.E mock Examinations, Despite all the tight Cirmumstances you still pushed through I am very proud of you I believe you will ace all subjects next Session </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Congratulations !!!!! For the Conlusion of your Second term/B.E.C.E mock Examinations, you have done it again Ayoka, it seems being at the top is now your portion, to be very honest with you, my only advice is for you to be "RELENTLESS" Don’t Stop working , the sky is just your Own Beginning not your limit </t>
+  </si>
+  <si>
+    <t>Congratulations !!!!! For the Conlusion of your Second term/B.E.C.E mock Examinations I am very proud you Abdulsamad this  result is a true reflection your Hardwork , it's  better you not to relent, keep Burning your Midnight Candle, in Every Positive thing you do towards your Academics Be Passionate with it and don't ever give up you might get tired but do not back down.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -168,9 +185,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -495,7 +513,7 @@
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="12.36328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.36328125" customWidth="1"/>
-    <col min="8" max="8" width="70.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="107.1796875" customWidth="1"/>
     <col min="10" max="10" width="11.90625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10.08984375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="9.7265625" bestFit="1" customWidth="1"/>
@@ -509,19 +527,19 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>21</v>
-      </c>
-      <c r="G1" t="s">
-        <v>22</v>
       </c>
       <c r="H1" t="s">
         <v>2</v>
@@ -553,43 +571,46 @@
         <v>23001</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D2">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E2">
-        <v>99</v>
+        <v>61</v>
+      </c>
+      <c r="F2">
+        <v>6</v>
       </c>
       <c r="G2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="H2" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="I2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="J2" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O2">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.35">
@@ -597,43 +618,46 @@
         <v>23002</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D3">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E3">
-        <v>99</v>
+        <v>62</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
       </c>
       <c r="G3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="H3" t="s">
-        <v>10</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="K3">
         <v>5</v>
       </c>
       <c r="L3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O3">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.35">
@@ -641,43 +665,46 @@
         <v>23003</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D4">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E4">
-        <v>99</v>
+        <v>62</v>
+      </c>
+      <c r="F4">
+        <v>5</v>
       </c>
       <c r="G4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="H4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="K4">
         <v>5</v>
       </c>
       <c r="L4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O4">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.35">
@@ -685,28 +712,31 @@
         <v>23004</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5">
+        <v>67</v>
+      </c>
+      <c r="E5">
+        <v>66</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" t="s">
         <v>35</v>
       </c>
-      <c r="D5">
-        <v>100</v>
-      </c>
-      <c r="E5">
-        <v>99</v>
-      </c>
-      <c r="G5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>28</v>
+      <c r="I5" t="s">
+        <v>24</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="K5">
         <v>5</v>
@@ -715,13 +745,13 @@
         <v>4</v>
       </c>
       <c r="M5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O5">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.35">
@@ -729,28 +759,31 @@
         <v>23005</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D6">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E6">
-        <v>99</v>
+        <v>61</v>
+      </c>
+      <c r="F6">
+        <v>6</v>
       </c>
       <c r="G6" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="H6" t="s">
-        <v>10</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
+      </c>
+      <c r="I6" t="s">
+        <v>24</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K6">
         <v>5</v>
@@ -759,13 +792,13 @@
         <v>4</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O6">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.35">
@@ -773,28 +806,31 @@
         <v>23008</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D7">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E7">
-        <v>99</v>
+        <v>66</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="H7" t="s">
-        <v>10</v>
-      </c>
-      <c r="I7" s="1" t="s">
         <v>31</v>
       </c>
+      <c r="I7" t="s">
+        <v>24</v>
+      </c>
       <c r="J7" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="K7">
         <v>5</v>
@@ -803,13 +839,13 @@
         <v>4</v>
       </c>
       <c r="M7">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O7">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
@@ -817,43 +853,46 @@
         <v>23006</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D8">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E8">
-        <v>99</v>
+        <v>66</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
       </c>
       <c r="G8" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" t="s">
+        <v>37</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="H8" t="s">
-        <v>10</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="K8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O8">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">
@@ -861,28 +900,31 @@
         <v>23007</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D9">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E9">
-        <v>99</v>
+        <v>66</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
       </c>
       <c r="G9" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="H9" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="K9">
         <v>5</v>
@@ -891,13 +933,13 @@
         <v>4</v>
       </c>
       <c r="M9">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O9">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.35">

</xml_diff>